<commit_message>
Tighten Sugar News supply-demand wording
</commit_message>
<xml_diff>
--- a/reports/2026/08/Sugar News 2026-08-04.xlsx
+++ b/reports/2026/08/Sugar News 2026-08-04.xlsx
@@ -530,7 +530,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>印度政府发布或调整乙醇掺混或燃料政策，关键数据包括E20。若新增乙醇需求由B重糖蜜、糖浆或甘蔗汁满足，糖厂会把这些可发酵糖源送入乙醇装置；其中B重糖蜜、糖浆和甘蔗汁会减少可结晶成白糖的蔗糖量。来源：The Times of India（https://news.google.com/rss/articles/CBMi8AFBVV95cUxOTS0tZVZFa09CZFptVzNQazAyX2pFOTFadkhobkt1VDdvTFZxRnhBVENuZjJhWFFFUnJneE1jRXF2TEo2b2EtVlRlVEpWY2ZZeHFNWEJGUE5pWWJ0Z0MzR1NwbnZXb0FURGRRZk5qUWdxdkFYYVdJbzVRekdudDNIX2ROaWRIcEVkTFpPd2QtSVYzazdnMXVLR0NjV3ZoRzI2UUt3WDl5emZUV1JhUmduRDI2T2ZYbWJJWTRwdkdNLV8wNFcyT1NRcnBWcTFUWDgxTjVFUWxTTktrYjlwUVkzSjdsbm5VTFAzUDU0YkE5bVXSAfABQVVfeXFMTk0tLWVWRWtPQmRabVczUGswMl9qRTkxWnZIaG5LdVQ3b0xWcUZ4QVRDbmYyYVhRRVJyZ3hNY0VxdkxKNm9hLVZUZVRKVmNmWXhxTVhCRlBOaVlidGdDM0dTcG52V29BVERkUWZOalFncXZBWGFXSW81UXpHbnQzSF9kTmlkSHBFZExaT3dkLUlWM2s3ZzF1S0dDY1d2aEcyNlFLd1g5eXpmVFdSYVJnbkQyNk9mWG1iSVk0cHZHTS1fMDRXMk9TUXJwVnExVFg4MU41RVFsU05La2I5cFFZM0o3bG5uVUxQM1A1NGJBOW1V?oc=5）</t>
+          <t>印度政府发布或调整E20乙醇掺混政策，掺混目标为E20。若新增乙醇需求由B重糖蜜、糖浆或甘蔗汁满足，糖厂会把这些可发酵糖源送入乙醇装置；其中B重糖蜜、糖浆和甘蔗汁会减少可结晶成白糖的蔗糖量。来源：The Times of India（https://news.google.com/rss/articles/CBMi8AFBVV95cUxOTS0tZVZFa09CZFptVzNQazAyX2pFOTFadkhobkt1VDdvTFZxRnhBVENuZjJhWFFFUnJneE1jRXF2TEo2b2EtVlRlVEpWY2ZZeHFNWEJGUE5pWWJ0Z0MzR1NwbnZXb0FURGRRZk5qUWdxdkFYYVdJbzVRekdudDNIX2ROaWRIcEVkTFpPd2QtSVYzazdnMXVLR0NjV3ZoRzI2UUt3WDl5emZUV1JhUmduRDI2T2ZYbWJJWTRwdkdNLV8wNFcyT1NRcnBWcTFUWDgxTjVFUWxTTktrYjlwUVkzSjdsbm5VTFAzUDU0YkE5bVXSAfABQVVfeXFMTk0tLWVWRWtPQmRabVczUGswMl9qRTkxWnZIaG5LdVQ3b0xWcUZ4QVRDbmYyYVhRRVJyZ3hNY0VxdkxKNm9hLVZUZVRKVmNmWXhxTVhCRlBOaVlidGdDM0dTcG52V29BVERkUWZOalFncXZBWGFXSW81UXpHbnQzSF9kTmlkSHBFZExaT3dkLUlWM2s3ZzF1S0dDY1d2aEcyNlFLd1g5eXpmVFdSYVJnbkQyNk9mWG1iSVk0cHZHTS1fMDRXMk9TUXJwVnExVFg4MU41RVFsU05La2I5cFFZM0o3bG5uVUxQM1A1NGJBOW1V?oc=5）</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -581,12 +581,12 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>菲律宾糖业相关机构公布食糖产量、库存、销量或消费预测，关键数据包括10.98%。产量、库存、销量或消费变化会直接改变食糖供需平衡。来源：manilatimes.net（https://news.google.com/rss/articles/CBMirgFBVV95cUxONWZYV3FLYkc1bjNFUEZlNWhMajZ4cnR0WHdtTENKMXZualZBOGtqZmtrNmRyVWZCMDc5Q2JvSmpIbHVjbmRQbXpCSzhMODVtQ3ktWFRYcVprRnBwWlBPR2pWU0xhcWhWMGo5MC1OdWdTdnNfZ0pKSGNUTDg3RWstalowWWk2d0JKZUJoVS1NN0lBQm10aUFRUWJVSDFWcjg4U2RYd1FJRXYxU01OdWfSAbMBQVVfeXFMUEJ3Q19aRDkzZ3pOQXVmaHltRXA3Tk5kUThsNDlwMnc1T2g4NU85eW5zUTR1cGNkZ2V1QWIzQ3I2ZXdEV2sxUl9OVjFHZ0JtbmtweEs3UVMyVDFETXB5MEZENHZsNFM4ZU1wNHRtVm9tNzNXNlJnVUxLakw5djlXd3BaM3VOVFBxYkZfTFZNYnFRRGx6QVdobjVIMy1OVDJGY1E5MWV1MXZ2SFdxdy1IZnpHa1k?oc=5）</t>
+          <t>菲律宾糖业监管署SRA公布糖产量数据，截至7月12日糖产量下降10.98%至185万吨。糖产量下降会减少当期新增可售糖源，收紧供应端并支撑糖价。来源：manilatimes.net（https://news.google.com/rss/articles/CBMirgFBVV95cUxONWZYV3FLYkc1bjNFUEZlNWhMajZ4cnR0WHdtTENKMXZualZBOGtqZmtrNmRyVWZCMDc5Q2JvSmpIbHVjbmRQbXpCSzhMODVtQ3ktWFRYcVprRnBwWlBPR2pWU0xhcWhWMGo5MC1OdWdTdnNfZ0pKSGNUTDg3RWstalowWWk2d0JKZUJoVS1NN0lBQm10aUFRUWJVSDFWcjg4U2RYd1FJRXYxU01OdWfSAbMBQVVfeXFMUEJ3Q19aRDkzZ3pOQXVmaHltRXA3Tk5kUThsNDlwMnc1T2g4NU85eW5zUTR1cGNkZ2V1QWIzQ3I2ZXdEV2sxUl9OVjFHZ0JtbmtweEs3UVMyVDFETXB5MEZENHZsNFM4ZU1wNHRtVm9tNzNXNlJnVUxLakw5djlXd3BaM3VOVFBxYkZfTFZNYnFRRGx6QVdobjVIMy1OVDJGY1E5MWV1MXZ2SFdxdy1IZnpHa1k?oc=5）</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>利多：产量下降、库存收缩或供应缺口会减少可用糖源并支撑糖价。</t>
+          <t>利多：糖产量下降会减少当期新增可售糖源，收紧供应端并支撑糖价。</t>
         </is>
       </c>
     </row>
@@ -615,12 +615,12 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>菲律宾主产区农业或气象机构预警甘蔗产区天气、干旱或病虫害，关键数据包括77.3 hectares。产区天气或病虫害变化会影响甘蔗生长、收割和糖料供应稳定性。来源：Digicast Negros（https://news.google.com/rss/articles/CBMi1gFBVV95cUxOcmtWNXBXMUw4ZWVPSEVpT3pWU3VlS2Z1a2xxLXFPLWVTMG1Ubk5NLUlJc2l1WEZKb25Makk5Z3JNVXhhLTgyS09WMk1rbXRmbXlwV0RBMHBWdnh0REtvV3A2akd3N1JOVGU2T1ZJaEdNTFRzY1BJaUMzMV9Mb3MxN3BFMGRoTUJENnJDUkpxc2k4RWc4QW51SWNTNm14bFVleVIxMzlucnBqYWdMNEtrZmdUd002bE9HemtBbklDbndyRUZJQlhzNFgwdVBJQkpMeXNpMWtB0gHWAUFVX3lxTE5ya1Y1cFcxTDhlZU9IRWlPelZTdWVLZnVrbHEtcU8tZVMwbVRuTk0tSUlzaXVYRkpvbkxqSTlnck1VeGEtODJLT1YyTWttdGZteXBXREEwcFZ2eHRES29XcDZqR3c3Uk5UZTZPVkloR01MVHNjUElpQzMxX0xvczE3cEUwZGhNQkQ2ckNSSnFzaThFZzhBbnVJY1M2bXhsVWV5UjEzOW5ycGphZ0w0S2tmZ1R3TTZsT0d6a0FuSUNud3JFRklCWHM0WDB1UElCSkx5c2kxa0E?oc=5）</t>
+          <t>菲律宾西内格罗斯省防控工作组使用真菌处理77.3公顷甘蔗病虫害地块，并计划扩大至3个地方政府辖区。病虫害防控扩大可降低甘蔗受害面积继续扩张的风险，但当前仍反映西内格罗斯蔗区病虫害压力，对糖料供应稳定性偏多糖价。来源：Digicast Negros（https://news.google.com/rss/articles/CBMi1gFBVV95cUxOcmtWNXBXMUw4ZWVPSEVpT3pWU3VlS2Z1a2xxLXFPLWVTMG1Ubk5NLUlJc2l1WEZKb25Makk5Z3JNVXhhLTgyS09WMk1rbXRmbXlwV0RBMHBWdnh0REtvV3A2akd3N1JOVGU2T1ZJaEdNTFRzY1BJaUMzMV9Mb3MxN3BFMGRoTUJENnJDUkpxc2k4RWc4QW51SWNTNm14bFVleVIxMzlucnBqYWdMNEtrZmdUd002bE9HemtBbklDbndyRUZJQlhzNFgwdVBJQkpMeXNpMWtB0gHWAUFVX3lxTE5ya1Y1cFcxTDhlZU9IRWlPelZTdWVLZnVrbHEtcU8tZVMwbVRuTk0tSUlzaXVYRkpvbkxqSTlnck1VeGEtODJLT1YyTWttdGZteXBXREEwcFZ2eHRES29XcDZqR3c3Uk5UZTZPVkloR01MVHNjUElpQzMxX0xvczE3cEUwZGhNQkQ2ckNSSnFzaThFZzhBbnVJY1M2bXhsVWV5UjEzOW5ycGphZ0w0S2tmZ1R3TTZsT0d6a0FuSUNud3JFRklCWHM0WDB1UElCSkx5c2kxa0E?oc=5）</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>利多：干旱、洪涝或病虫害会压低甘蔗单产并削弱糖料供应稳定性，从而支撑糖价。</t>
+          <t>利多：病虫害已需在77.3公顷地块进行防控，说明西内格罗斯蔗区糖料供应存在单产风险，若扩散会减少可入榨甘蔗并支撑糖价。</t>
         </is>
       </c>
     </row>

</xml_diff>